<commit_message>
Tracker re-checked against production, 25 Sep 2026
Point 24 (manager KRA edit) is closed, so the 31-point list stands at
22 completed / 9 pending. Point 22's note now records the two logins
that actually exist on production and that a manager login with reports
is still missing. New "After the 31 points" tab lists the 26 items
raised on 23-24 Sep, all built and deployed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RhX1xUA47iJu7ozfwA1Vhh
</commit_message>
<xml_diff>
--- a/docs/Agentic-PMS-31-point-tracker.xlsx
+++ b/docs/Agentic-PMS-31-point-tracker.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What we need from you" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="After the 31 points" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What we need from you" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tracker'!$A$4:$L$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$4:$L$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,6 +93,31 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -157,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -246,6 +272,26 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -656,7 +702,7 @@
     <row r="2">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Snapshot of the Tracker tab as it stood on 24 Sep 2026, checked against the code deployed to production (commit ad934fc). 21 completed, 10 pending. The Tracker tab carries the detail and the evidence for each row.</t>
+          <t>Re-checked on 25 Sep 2026 against the code deployed to production (commit f0b36bd, 52 migrations) and against the production database. 22 completed, 9 pending. The Tracker tab carries the detail and the evidence for each row; the "After the 31 points" tab lists the work raised since this list was drawn up.</t>
         </is>
       </c>
     </row>
@@ -667,7 +713,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="32" t="n"/>
       <c r="D4" s="32" t="n"/>
@@ -680,7 +726,7 @@
         </is>
       </c>
       <c r="B5" s="31" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" s="32" t="n"/>
       <c r="D5" s="32" t="n"/>
@@ -726,612 +772,612 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="34" t="n">
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="43" t="n">
         <v>1</v>
       </c>
-      <c r="B9" s="35" t="inlineStr">
+      <c r="B9" s="44" t="inlineStr">
         <is>
           <t>Approved goals: remove the edit lock</t>
         </is>
       </c>
-      <c r="C9" s="36" t="inlineStr">
+      <c r="C9" s="45" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D9" s="35" t="inlineStr">
-        <is>
-          <t>Decide: should an approved growth plan be directly editable, or keep 'ask your manager to return it'?</t>
-        </is>
-      </c>
-      <c r="E9" s="35" t="inlineStr">
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>Decide: should an approved growth plan be directly editable, or keep 'ask your manager to return it'? Still locked in the deployed build.</t>
+        </is>
+      </c>
+      <c r="E9" s="44" t="inlineStr">
         <is>
           <t>Mindgate — decision</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="34" t="n">
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="43" t="n">
         <v>2</v>
       </c>
-      <c r="B10" s="35" t="inlineStr">
+      <c r="B10" s="44" t="inlineStr">
         <is>
           <t>Department dropdown for KRA setup</t>
         </is>
       </c>
-      <c r="C10" s="36" t="inlineStr">
+      <c r="C10" s="45" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D10" s="35" t="inlineStr">
-        <is>
-          <t>Add a Department value to the library rows and re-publish the sheet.</t>
-        </is>
-      </c>
-      <c r="E10" s="35" t="inlineStr">
+      <c r="D10" s="44" t="inlineStr">
+        <is>
+          <t>Add a Department value to the library rows and re-publish the sheet. Checked 25 Sep: 0 of the 2,155 library rows carries a department.</t>
+        </is>
+      </c>
+      <c r="E10" s="44" t="inlineStr">
         <is>
           <t>Mindgate — data</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="34" t="n">
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="43" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="35" t="inlineStr">
+      <c r="B11" s="44" t="inlineStr">
         <is>
           <t>KRA unique ID</t>
         </is>
       </c>
-      <c r="C11" s="36" t="inlineStr">
+      <c r="C11" s="45" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D11" s="35" t="inlineStr">
-        <is>
-          <t>Answer: (a) format, e.g. SALES-SM-001; (b) unique per library row or per assigned KRA; (c) does the ID change when the KRA is edited or re-mapped; (d) what happens to the 2,155 rows already loaded.</t>
-        </is>
-      </c>
-      <c r="E11" s="35" t="inlineStr">
+      <c r="D11" s="44" t="inlineStr">
+        <is>
+          <t>Answer: (a) format, e.g. SALES-SM-001; (b) unique per library row or per assigned KRA; (c) does the ID change when the KRA is edited or re-mapped; (d) what happens to the IDs already assigned. No ID field exists yet.</t>
+        </is>
+      </c>
+      <c r="E11" s="44" t="inlineStr">
         <is>
           <t>Mindgate — decision</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="34" t="n">
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="43" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="35" t="inlineStr">
+      <c r="B12" s="44" t="inlineStr">
         <is>
           <t>Google Meet integration</t>
         </is>
       </c>
-      <c r="C12" s="36" t="inlineStr">
+      <c r="C12" s="45" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D12" s="35" t="inlineStr">
-        <is>
-          <t>Provide Google OAuth client ID and secret for the workspace.</t>
-        </is>
-      </c>
-      <c r="E12" s="35" t="inlineStr">
+      <c r="D12" s="44" t="inlineStr">
+        <is>
+          <t>Provide Google OAuth client ID and secret for the workspace. Not configured on the box as of 25 Sep.</t>
+        </is>
+      </c>
+      <c r="E12" s="44" t="inlineStr">
         <is>
           <t>Mindgate — credentials</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="34" t="n">
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="43" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="35" t="inlineStr">
+      <c r="B13" s="44" t="inlineStr">
         <is>
           <t>RM approval issue</t>
         </is>
       </c>
-      <c r="C13" s="36" t="inlineStr">
+      <c r="C13" s="45" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D13" s="35" t="inlineStr">
-        <is>
-          <t>Comes free with point 22.</t>
-        </is>
-      </c>
-      <c r="E13" s="35" t="inlineStr">
+      <c r="D13" s="44" t="inlineStr">
+        <is>
+          <t>Comes free with point 22. The approve path itself works and is tested; no manager with reports can sign in to exercise it.</t>
+        </is>
+      </c>
+      <c r="E13" s="44" t="inlineStr">
         <is>
           <t>Mindgate — accounts</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="34" t="n">
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="43" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="35" t="inlineStr">
+      <c r="B14" s="44" t="inlineStr">
         <is>
           <t>KRA synchronisation</t>
         </is>
       </c>
-      <c r="C14" s="36" t="inlineStr">
+      <c r="C14" s="45" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D14" s="35" t="inlineStr">
-        <is>
-          <t>Same as point 2.</t>
-        </is>
-      </c>
-      <c r="E14" s="35" t="inlineStr">
+      <c r="D14" s="44" t="inlineStr">
+        <is>
+          <t>Same as point 2 — the department values on the library rows.</t>
+        </is>
+      </c>
+      <c r="E14" s="44" t="inlineStr">
         <is>
           <t>Mindgate — data</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="34" t="n">
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="43" t="n">
         <v>17</v>
       </c>
-      <c r="B15" s="35" t="inlineStr">
+      <c r="B15" s="44" t="inlineStr">
         <is>
           <t>Quarterly Connect email</t>
         </is>
       </c>
-      <c r="C15" s="36" t="inlineStr">
+      <c r="C15" s="45" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D15" s="35" t="inlineStr">
-        <is>
-          <t>Provide SMTP host, port, user and password.</t>
-        </is>
-      </c>
-      <c r="E15" s="35" t="inlineStr">
+      <c r="D15" s="44" t="inlineStr">
+        <is>
+          <t>Provide SMTP host, port, user and password. Still unset on production, so no mail leaves the box.</t>
+        </is>
+      </c>
+      <c r="E15" s="44" t="inlineStr">
         <is>
           <t>Mindgate — credentials</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="34" t="n">
+    <row r="16" ht="44" customHeight="1">
+      <c r="A16" s="43" t="n">
         <v>22</v>
       </c>
-      <c r="B16" s="35" t="inlineStr">
+      <c r="B16" s="44" t="inlineStr">
         <is>
           <t>Access setup for testing</t>
         </is>
       </c>
-      <c r="C16" s="36" t="inlineStr">
+      <c r="C16" s="45" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D16" s="35" t="inlineStr">
-        <is>
-          <t>Create one employee and one manager login on production. Minutes of work; blocks points 7, 24, 25, 26 being tested by you.</t>
-        </is>
-      </c>
-      <c r="E16" s="35" t="inlineStr">
+      <c r="D16" s="44" t="inlineStr">
+        <is>
+          <t>Create one manager login — somebody who actually has reports. Production has only two logins today (hr.admin@mindgate.com and pavan.kumar@mindgate.in, 0 reports). That one account unblocks point 7.</t>
+        </is>
+      </c>
+      <c r="E16" s="44" t="inlineStr">
         <is>
           <t>Us — needs your go-ahead</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="34" t="n">
+    <row r="17" ht="44" customHeight="1">
+      <c r="A17" s="43" t="n">
+        <v>31</v>
+      </c>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t>Quarterly connect should focus more on confirmation</t>
+        </is>
+      </c>
+      <c r="C17" s="45" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="D17" s="44" t="inlineStr">
+        <is>
+          <t>Tell us what 'more confirmation' means beyond the sign-off that already exists. Adding pending sign-offs to All Approvals is small and we can do it now.</t>
+        </is>
+      </c>
+      <c r="E17" s="44" t="inlineStr">
+        <is>
+          <t>Mindgate — clarify</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t>Associate the growth path after the KRA</t>
+        </is>
+      </c>
+      <c r="C18" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D18" s="44" t="inlineStr">
+        <is>
+          <t>Tell us what 'more confirmation' means beyond sign-off. Adding pending sign-offs to All Approvals is small and we can do it now.</t>
+        </is>
+      </c>
+      <c r="E18" s="44" t="inlineStr">
+        <is>
+          <t>Mindgate — clarify</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t>KRAs always open + new-hire auto-assign</t>
+        </is>
+      </c>
+      <c r="C19" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D19" s="44" t="inlineStr"/>
+      <c r="E19" s="44" t="inlineStr"/>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY missing in My Growth</t>
+        </is>
+      </c>
+      <c r="C20" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D20" s="44" t="inlineStr"/>
+      <c r="E20" s="44" t="inlineStr"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="43" t="n">
+        <v>9</v>
+      </c>
+      <c r="B21" s="44" t="inlineStr">
+        <is>
+          <t>KRA Library editing</t>
+        </is>
+      </c>
+      <c r="C21" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D21" s="44" t="inlineStr"/>
+      <c r="E21" s="44" t="inlineStr"/>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="B22" s="44" t="inlineStr">
+        <is>
+          <t>Role / department change</t>
+        </is>
+      </c>
+      <c r="C22" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D22" s="44" t="inlineStr"/>
+      <c r="E22" s="44" t="inlineStr"/>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="43" t="n">
+        <v>11</v>
+      </c>
+      <c r="B23" s="44" t="inlineStr">
+        <is>
+          <t>'Select all KRAs' in My Growth</t>
+        </is>
+      </c>
+      <c r="C23" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D23" s="44" t="inlineStr"/>
+      <c r="E23" s="44" t="inlineStr"/>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="43" t="n">
+        <v>13</v>
+      </c>
+      <c r="B24" s="44" t="inlineStr">
+        <is>
+          <t>Career pathing matrix under Aspiring Career</t>
+        </is>
+      </c>
+      <c r="C24" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D24" s="44" t="inlineStr"/>
+      <c r="E24" s="44" t="inlineStr"/>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="43" t="n">
+        <v>14</v>
+      </c>
+      <c r="B25" s="44" t="inlineStr">
+        <is>
+          <t>Career pathing template</t>
+        </is>
+      </c>
+      <c r="C25" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D25" s="44" t="inlineStr"/>
+      <c r="E25" s="44" t="inlineStr"/>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="43" t="n">
+        <v>15</v>
+      </c>
+      <c r="B26" s="44" t="inlineStr">
+        <is>
+          <t>Department management</t>
+        </is>
+      </c>
+      <c r="C26" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D26" s="44" t="inlineStr"/>
+      <c r="E26" s="44" t="inlineStr"/>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="43" t="n">
+        <v>16</v>
+      </c>
+      <c r="B27" s="44" t="inlineStr">
+        <is>
+          <t>Mid-year self-appraisal</t>
+        </is>
+      </c>
+      <c r="C27" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D27" s="44" t="inlineStr"/>
+      <c r="E27" s="44" t="inlineStr"/>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="43" t="n">
+        <v>18</v>
+      </c>
+      <c r="B28" s="44" t="inlineStr">
+        <is>
+          <t>Rename Self-Appraisal to Annual Review</t>
+        </is>
+      </c>
+      <c r="C28" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D28" s="44" t="inlineStr"/>
+      <c r="E28" s="44" t="inlineStr"/>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="43" t="n">
+        <v>19</v>
+      </c>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Rename Annual Review to Final Rating</t>
+        </is>
+      </c>
+      <c r="C29" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D29" s="44" t="inlineStr"/>
+      <c r="E29" s="44" t="inlineStr"/>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="43" t="n">
+        <v>20</v>
+      </c>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Manager rating visibility</t>
+        </is>
+      </c>
+      <c r="C30" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D30" s="44" t="inlineStr"/>
+      <c r="E30" s="44" t="inlineStr"/>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="43" t="n">
+        <v>21</v>
+      </c>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Final rating publishing rights</t>
+        </is>
+      </c>
+      <c r="C31" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D31" s="44" t="inlineStr"/>
+      <c r="E31" s="44" t="inlineStr"/>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="43" t="n">
+        <v>23</v>
+      </c>
+      <c r="B32" s="44" t="inlineStr">
+        <is>
+          <t>Global search and approval buttons</t>
+        </is>
+      </c>
+      <c r="C32" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D32" s="44" t="inlineStr"/>
+      <c r="E32" s="44" t="inlineStr"/>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="43" t="n">
         <v>24</v>
       </c>
-      <c r="B17" s="35" t="inlineStr">
+      <c r="B33" s="44" t="inlineStr">
         <is>
           <t>KRA approval workflow</t>
         </is>
       </c>
-      <c r="C17" s="36" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D17" s="35" t="inlineStr">
-        <is>
-          <t>Decide whether a manager may edit a report's KRA sheet during review. If yes, we add edit + Save &amp; Submit to the manager review card. Half a day.</t>
-        </is>
-      </c>
-      <c r="E17" s="35" t="inlineStr">
-        <is>
-          <t>Us</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="34" t="n">
-        <v>31</v>
-      </c>
-      <c r="B18" s="35" t="inlineStr">
-        <is>
-          <t>Quarterly connect should focus more on confirmation</t>
-        </is>
-      </c>
-      <c r="C18" s="36" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D18" s="35" t="inlineStr">
-        <is>
-          <t>Tell us what 'more confirmation' means beyond sign-off. Adding pending sign-offs to All Approvals is small and we can do it now.</t>
-        </is>
-      </c>
-      <c r="E18" s="35" t="inlineStr">
-        <is>
-          <t>Mindgate — clarify</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="34" t="n">
-        <v>3</v>
-      </c>
-      <c r="B19" s="35" t="inlineStr">
-        <is>
-          <t>Associate the growth path after the KRA</t>
-        </is>
-      </c>
-      <c r="C19" s="37" t="inlineStr">
+      <c r="C33" s="46" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="D19" s="35" t="inlineStr"/>
-      <c r="E19" s="35" t="inlineStr"/>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="34" t="n">
-        <v>6</v>
-      </c>
-      <c r="B20" s="35" t="inlineStr">
-        <is>
-          <t>KRAs always open + new-hire auto-assign</t>
-        </is>
-      </c>
-      <c r="C20" s="37" t="inlineStr">
+      <c r="D33" s="44" t="inlineStr"/>
+      <c r="E33" s="44" t="inlineStr"/>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="43" t="n">
+        <v>25</v>
+      </c>
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Role-based views</t>
+        </is>
+      </c>
+      <c r="C34" s="46" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="D20" s="35" t="inlineStr"/>
-      <c r="E20" s="35" t="inlineStr"/>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="34" t="n">
-        <v>8</v>
-      </c>
-      <c r="B21" s="35" t="inlineStr">
-        <is>
-          <t>ANTHROPIC_API_KEY missing in My Growth</t>
-        </is>
-      </c>
-      <c r="C21" s="37" t="inlineStr">
+      <c r="D34" s="44" t="inlineStr"/>
+      <c r="E34" s="44" t="inlineStr"/>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="43" t="n">
+        <v>26</v>
+      </c>
+      <c r="B35" s="44" t="inlineStr">
+        <is>
+          <t>Manager dashboard tracking</t>
+        </is>
+      </c>
+      <c r="C35" s="46" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="D21" s="35" t="inlineStr"/>
-      <c r="E21" s="35" t="inlineStr"/>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="34" t="n">
-        <v>9</v>
-      </c>
-      <c r="B22" s="35" t="inlineStr">
-        <is>
-          <t>KRA Library editing</t>
-        </is>
-      </c>
-      <c r="C22" s="37" t="inlineStr">
+      <c r="D35" s="44" t="inlineStr"/>
+      <c r="E35" s="44" t="inlineStr"/>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="43" t="n">
+        <v>27</v>
+      </c>
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analytics dashboard on login</t>
+        </is>
+      </c>
+      <c r="C36" s="46" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="D22" s="35" t="inlineStr"/>
-      <c r="E22" s="35" t="inlineStr"/>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="34" t="n">
-        <v>10</v>
-      </c>
-      <c r="B23" s="35" t="inlineStr">
-        <is>
-          <t>Role / department change</t>
-        </is>
-      </c>
-      <c r="C23" s="37" t="inlineStr">
+      <c r="D36" s="44" t="inlineStr"/>
+      <c r="E36" s="44" t="inlineStr"/>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="43" t="n">
+        <v>28</v>
+      </c>
+      <c r="B37" s="44" t="inlineStr">
+        <is>
+          <t>UI does not match the shared screens</t>
+        </is>
+      </c>
+      <c r="C37" s="46" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="D23" s="35" t="inlineStr"/>
-      <c r="E23" s="35" t="inlineStr"/>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="34" t="n">
-        <v>11</v>
-      </c>
-      <c r="B24" s="35" t="inlineStr">
-        <is>
-          <t>'Select all KRAs' in My Growth</t>
-        </is>
-      </c>
-      <c r="C24" s="37" t="inlineStr">
+      <c r="D37" s="44" t="inlineStr"/>
+      <c r="E37" s="44" t="inlineStr"/>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="43" t="n">
+        <v>29</v>
+      </c>
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>Current designation in the growth section</t>
+        </is>
+      </c>
+      <c r="C38" s="46" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="D24" s="35" t="inlineStr"/>
-      <c r="E24" s="35" t="inlineStr"/>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="34" t="n">
-        <v>13</v>
-      </c>
-      <c r="B25" s="35" t="inlineStr">
-        <is>
-          <t>Career pathing matrix under Aspiring Career</t>
-        </is>
-      </c>
-      <c r="C25" s="37" t="inlineStr">
+      <c r="D38" s="44" t="inlineStr"/>
+      <c r="E38" s="44" t="inlineStr"/>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="43" t="n">
+        <v>30</v>
+      </c>
+      <c r="B39" s="44" t="inlineStr">
+        <is>
+          <t>Potential rating + mid-year checkpoint</t>
+        </is>
+      </c>
+      <c r="C39" s="46" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="D25" s="35" t="inlineStr"/>
-      <c r="E25" s="35" t="inlineStr"/>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="34" t="n">
-        <v>14</v>
-      </c>
-      <c r="B26" s="35" t="inlineStr">
-        <is>
-          <t>Career pathing template</t>
-        </is>
-      </c>
-      <c r="C26" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D26" s="35" t="inlineStr"/>
-      <c r="E26" s="35" t="inlineStr"/>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="34" t="n">
-        <v>15</v>
-      </c>
-      <c r="B27" s="35" t="inlineStr">
-        <is>
-          <t>Department management</t>
-        </is>
-      </c>
-      <c r="C27" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D27" s="35" t="inlineStr"/>
-      <c r="E27" s="35" t="inlineStr"/>
-    </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="34" t="n">
-        <v>16</v>
-      </c>
-      <c r="B28" s="35" t="inlineStr">
-        <is>
-          <t>Mid-year self-appraisal</t>
-        </is>
-      </c>
-      <c r="C28" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D28" s="35" t="inlineStr"/>
-      <c r="E28" s="35" t="inlineStr"/>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="34" t="n">
-        <v>18</v>
-      </c>
-      <c r="B29" s="35" t="inlineStr">
-        <is>
-          <t>Rename Self-Appraisal to Annual Review</t>
-        </is>
-      </c>
-      <c r="C29" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D29" s="35" t="inlineStr"/>
-      <c r="E29" s="35" t="inlineStr"/>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="34" t="n">
-        <v>19</v>
-      </c>
-      <c r="B30" s="35" t="inlineStr">
-        <is>
-          <t>Rename Annual Review to Final Rating</t>
-        </is>
-      </c>
-      <c r="C30" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D30" s="35" t="inlineStr"/>
-      <c r="E30" s="35" t="inlineStr"/>
-    </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="34" t="n">
-        <v>20</v>
-      </c>
-      <c r="B31" s="35" t="inlineStr">
-        <is>
-          <t>Manager rating visibility</t>
-        </is>
-      </c>
-      <c r="C31" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D31" s="35" t="inlineStr"/>
-      <c r="E31" s="35" t="inlineStr"/>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="34" t="n">
-        <v>21</v>
-      </c>
-      <c r="B32" s="35" t="inlineStr">
-        <is>
-          <t>Final rating publishing rights</t>
-        </is>
-      </c>
-      <c r="C32" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D32" s="35" t="inlineStr"/>
-      <c r="E32" s="35" t="inlineStr"/>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="34" t="n">
-        <v>23</v>
-      </c>
-      <c r="B33" s="35" t="inlineStr">
-        <is>
-          <t>Global search and approval buttons</t>
-        </is>
-      </c>
-      <c r="C33" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D33" s="35" t="inlineStr"/>
-      <c r="E33" s="35" t="inlineStr"/>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="34" t="n">
-        <v>25</v>
-      </c>
-      <c r="B34" s="35" t="inlineStr">
-        <is>
-          <t>Role-based views</t>
-        </is>
-      </c>
-      <c r="C34" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D34" s="35" t="inlineStr"/>
-      <c r="E34" s="35" t="inlineStr"/>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="34" t="n">
-        <v>26</v>
-      </c>
-      <c r="B35" s="35" t="inlineStr">
-        <is>
-          <t>Manager dashboard tracking</t>
-        </is>
-      </c>
-      <c r="C35" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D35" s="35" t="inlineStr"/>
-      <c r="E35" s="35" t="inlineStr"/>
-    </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="34" t="n">
-        <v>27</v>
-      </c>
-      <c r="B36" s="35" t="inlineStr">
-        <is>
-          <t>Analytics dashboard on login</t>
-        </is>
-      </c>
-      <c r="C36" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D36" s="35" t="inlineStr"/>
-      <c r="E36" s="35" t="inlineStr"/>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="34" t="n">
-        <v>28</v>
-      </c>
-      <c r="B37" s="35" t="inlineStr">
-        <is>
-          <t>UI does not match the shared screens</t>
-        </is>
-      </c>
-      <c r="C37" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D37" s="35" t="inlineStr"/>
-      <c r="E37" s="35" t="inlineStr"/>
-    </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="34" t="n">
-        <v>29</v>
-      </c>
-      <c r="B38" s="35" t="inlineStr">
-        <is>
-          <t>Current designation in the growth section</t>
-        </is>
-      </c>
-      <c r="C38" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D38" s="35" t="inlineStr"/>
-      <c r="E38" s="35" t="inlineStr"/>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="34" t="n">
-        <v>30</v>
-      </c>
-      <c r="B39" s="35" t="inlineStr">
-        <is>
-          <t>Potential rating + mid-year checkpoint</t>
-        </is>
-      </c>
-      <c r="C39" s="37" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="D39" s="35" t="inlineStr"/>
-      <c r="E39" s="35" t="inlineStr"/>
+      <c r="D39" s="44" t="inlineStr"/>
+      <c r="E39" s="44" t="inlineStr"/>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="38" t="inlineStr">
@@ -1351,6 +1397,634 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>Everything asked for after the 31-point list</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>Every point raised on 23 and 24 Sep 2026. All of it is built, tested and live on production (commit f0b36bd). Nothing on this tab is waiting on us.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>What you asked for</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>Where it is</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="42" t="inlineStr">
+        <is>
+          <t>23 Sep</t>
+        </is>
+      </c>
+      <c r="B5" s="42" t="inlineStr">
+        <is>
+          <t>Engagement tab should be under HR, not My Performance</t>
+        </is>
+      </c>
+      <c r="C5" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D5" s="42" t="inlineStr">
+        <is>
+          <t>Split: My Surveys stays on Self; Engagement Surveys is on HR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="42" t="inlineStr">
+        <is>
+          <t>23 Sep</t>
+        </is>
+      </c>
+      <c r="B6" s="42" t="inlineStr">
+        <is>
+          <t>A better format for creating surveys</t>
+        </is>
+      </c>
+      <c r="C6" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D6" s="42" t="inlineStr">
+        <is>
+          <t>Survey builder rebuilt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="42" t="inlineStr">
+        <is>
+          <t>23 Sep</t>
+        </is>
+      </c>
+      <c r="B7" s="42" t="inlineStr">
+        <is>
+          <t>My Growth still shows team target achievements — move to Manager</t>
+        </is>
+      </c>
+      <c r="C7" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>Team Target Achievements is its own Manager page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="42" t="inlineStr">
+        <is>
+          <t>23 Sep</t>
+        </is>
+      </c>
+      <c r="B8" s="42" t="inlineStr">
+        <is>
+          <t>Mid-year under My Performance shows manager reviews — hide</t>
+        </is>
+      </c>
+      <c r="C8" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D8" s="42" t="inlineStr">
+        <is>
+          <t>Split into Team Mid-Year on the Manager tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="42" t="inlineStr">
+        <is>
+          <t>23 Sep</t>
+        </is>
+      </c>
+      <c r="B9" s="42" t="inlineStr">
+        <is>
+          <t>Remove the 7 parameters from all tabs</t>
+        </is>
+      </c>
+      <c r="C9" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D9" s="42" t="inlineStr">
+        <is>
+          <t>Grid and page removed; the annual rating now comes from the per-KRA weights.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="42" t="inlineStr">
+        <is>
+          <t>23 Sep</t>
+        </is>
+      </c>
+      <c r="B10" s="42" t="inlineStr">
+        <is>
+          <t>Return KRA option missing; KRA view not available</t>
+        </is>
+      </c>
+      <c r="C10" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D10" s="42" t="inlineStr">
+        <is>
+          <t>All Approvals expands each record and offers Approve / Return.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="42" t="inlineStr">
+        <is>
+          <t>23 Sep</t>
+        </is>
+      </c>
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t>Replace pink with blue everywhere</t>
+        </is>
+      </c>
+      <c r="C11" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Palette changed; a browser test reads the computed colours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B12" s="42" t="inlineStr">
+        <is>
+          <t>Export on Employees and the PMS Completion Report</t>
+        </is>
+      </c>
+      <c r="C12" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D12" s="42" t="inlineStr">
+        <is>
+          <t>.xlsx and .csv on both; employee codes keep their leading zeros.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B13" s="42" t="inlineStr">
+        <is>
+          <t>Make the KRA Overview counts clickable</t>
+        </is>
+      </c>
+      <c r="C13" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D13" s="42" t="inlineStr">
+        <is>
+          <t>Each count filters the table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B14" s="42" t="inlineStr">
+        <is>
+          <t>Search on Team Overview</t>
+        </is>
+      </c>
+      <c r="C14" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D14" s="42" t="inlineStr">
+        <is>
+          <t>Shared search control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B15" s="42" t="inlineStr">
+        <is>
+          <t>Team KRA Sheets / Evaluation / Mid-Year: only my reportees</t>
+        </is>
+      </c>
+      <c r="C15" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D15" s="42" t="inlineStr">
+        <is>
+          <t>Manager tab scoped to direct reports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t>KRA Library: clear previous data, add and delete a single KRA</t>
+        </is>
+      </c>
+      <c r="C16" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D16" s="42" t="inlineStr">
+        <is>
+          <t>Add sits beside Clear; clearing needs a typed confirmation and a matching count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Remove the "All employees" option from the Manager tab</t>
+        </is>
+      </c>
+      <c r="C17" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D17" s="42" t="inlineStr">
+        <is>
+          <t>Scope toggle deleted from all five pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t>A Manager dashboard like the Self one</t>
+        </is>
+      </c>
+      <c r="C18" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D18" s="42" t="inlineStr">
+        <is>
+          <t>Stat strip, action band, desk, named waiting-on-you list, roster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t>Fill the Career Pathing Matrix per department and designation</t>
+        </is>
+      </c>
+      <c r="C19" s="42" t="inlineStr">
+        <is>
+          <t>Done — needs your upload</t>
+        </is>
+      </c>
+      <c r="D19" s="42" t="inlineStr">
+        <is>
+          <t>159 transitions generated from the live master; "Download suggested matrix" on the page. 29 rows marked PLEASE CHECK. Not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B20" s="42" t="inlineStr">
+        <is>
+          <t>Competency mapping system — self and manager evaluation</t>
+        </is>
+      </c>
+      <c r="C20" s="42" t="inlineStr">
+        <is>
+          <t>Done — not yet used</t>
+        </is>
+      </c>
+      <c r="D20" s="42" t="inlineStr">
+        <is>
+          <t>Four screens from your workbook; 40 competencies seeded. 1 assessment started, 0 manager-submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="inlineStr">
+        <is>
+          <t>How the 9-box will display after competency mapping</t>
+        </is>
+      </c>
+      <c r="C21" s="42" t="inlineStr">
+        <is>
+          <t>Done — no data yet</t>
+        </is>
+      </c>
+      <c r="D21" s="42" t="inlineStr">
+        <is>
+          <t>Second view on the 9-box. Empty until annual ratings and manager competency ratings exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t>Super 50 — last 3 annual reviews, A or A+, this year A+</t>
+        </is>
+      </c>
+      <c r="C22" s="42" t="inlineStr">
+        <is>
+          <t>Done — needs history</t>
+        </is>
+      </c>
+      <c r="D22" s="42" t="inlineStr">
+        <is>
+          <t>Rule reads grades off the scale and is configurable. 0 published cycles and 0 prior years imported, so it cannot fire yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B23" s="42" t="inlineStr">
+        <is>
+          <t>Manager can edit a KRA after the employee submits</t>
+        </is>
+      </c>
+      <c r="C23" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>Edit on Team KRA Sheets; every change audited and the employee notified. Closes point 24 of the 31.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B24" s="42" t="inlineStr">
+        <is>
+          <t>Reporting manager change should move open KRAs</t>
+        </is>
+      </c>
+      <c r="C24" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D24" s="42" t="inlineStr">
+        <is>
+          <t>All five open record types move; submitted work stays with whoever wrote it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B25" s="42" t="inlineStr">
+        <is>
+          <t>Separate HOD tab, removed from Manager</t>
+        </is>
+      </c>
+      <c r="C25" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D25" s="42" t="inlineStr">
+        <is>
+          <t>Delivery Head is its own tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B26" s="42" t="inlineStr">
+        <is>
+          <t>Department dropdown on Team KRAs</t>
+        </is>
+      </c>
+      <c r="C26" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D26" s="42" t="inlineStr">
+        <is>
+          <t>Pick a department you staff or head; admins any.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B27" s="42" t="inlineStr">
+        <is>
+          <t>Suggestion of next appraisal</t>
+        </is>
+      </c>
+      <c r="C27" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D27" s="42" t="inlineStr">
+        <is>
+          <t>Each employee is told their own next appraisal on the cycle card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B28" s="42" t="inlineStr">
+        <is>
+          <t>Reminder to managers for pending approvals</t>
+        </is>
+      </c>
+      <c r="C28" s="42" t="inlineStr">
+        <is>
+          <t>Done — needs SMTP for email</t>
+        </is>
+      </c>
+      <c r="D28" s="42" t="inlineStr">
+        <is>
+          <t>In-app now. Email needs the SMTP credentials (point 17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B29" s="42" t="inlineStr">
+        <is>
+          <t>Appraisal eligibility by joining date</t>
+        </is>
+      </c>
+      <c r="C29" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>Both sentences on the cycle card with the real dates; configurable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="42" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B30" s="42" t="inlineStr">
+        <is>
+          <t>Ratings in alphabets, not numbers</t>
+        </is>
+      </c>
+      <c r="C30" s="42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D30" s="42" t="inlineStr">
+        <is>
+          <t>One formatter across every page, the exports and the closure-letter PDF.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1383,7 +2057,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Status checked against the code deployed to production (commit ad934fc) on 24 Sep 2026. The three data-dependent rows (2/12, 13, 22) are as last measured on the live box on 23 Sep — the instance is stopped at your request, so they were not re-probed. Columns I to L are yours to fill in; everything left of them is the check.</t>
+          <t>Status re-checked against the code deployed to production (commit f0b36bd, 52 migrations) and against the production database, on 25 Sep 2026.</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2994,7 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Only hr.admin@mindgate.com has a password. Roles held: 1 admin, 5 hod, 239 manager, 0 hr — but none of the managers can sign in.</t>
+          <t>Partly resolved. Two logins exist on production: hr.admin@mindgate.com (admin) and pavan.kumar@mindgate.in (employee role, 0 reports). There is still NO manager login with reports, so the manager approval path (point 7) cannot be exercised end to end.</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
@@ -2330,7 +3004,7 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>Create one employee and one manager login on production. Minutes of work; blocks points 7, 24, 25, 26 being tested by you.</t>
+          <t>Create one manager login — somebody who actually has reports. That alone unblocks point 7 and lets the full submit-approve loop be demonstrated.</t>
         </is>
       </c>
       <c r="H26" s="8" t="n">
@@ -2397,27 +3071,25 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Partly done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>DONE: the Approved tab exists (Pending your review / Approved / Returned / Not submitted), and approving an unchanged sheet is one click, on the manager page and on All Approvals. NOT DONE: "Save &amp; Submit when edited" — a MANAGER still cannot edit a report's sheet, only Approve or Return it for the employee to change. HR can edit and submit on someone's behalf from KRA Overview; the manager has no equivalent.</t>
+          <t>Closed 24 Sep 2026. A manager can now edit a submitted KRA sheet in place on Team KRA Sheets — submitted sheets only, weights must still total 100, every field change audited before/after, and the employee notified. The sheet stays submitted, so Approve/Return still apply.</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>Us</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>Decide whether a manager may edit a report's KRA sheet during review. If yes, we add edit + Save &amp; Submit to the manager review card. Half a day.</t>
-        </is>
-      </c>
-      <c r="H28" s="8" t="n">
-        <v>8</v>
-      </c>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="n"/>
       <c r="I28" s="10" t="inlineStr"/>
       <c r="J28" s="10" t="inlineStr"/>
       <c r="K28" s="8" t="inlineStr"/>
@@ -2714,7 +3386,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3012,7 +3684,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Close points 1, 2, 4, 7 and 12 on Mindgate's confirmation
Mindgate confirmed on 25 Sep that points 1, 2, 4 and 12 are resolved
through the department mapping and that point 7 (reporting-manager
approval) is working. Point 22 stays open — Mindgate is creating the
logins from their side.

The list now stands at 27 completed / 4 pending: Google OAuth (5), SMTP
(17), the test logins (22) and the quarterly-connect clarification (31).
Summary and "What we need from you" tabs updated to match.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RhX1xUA47iJu7ozfwA1Vhh
</commit_message>
<xml_diff>
--- a/docs/Agentic-PMS-31-point-tracker.xlsx
+++ b/docs/Agentic-PMS-31-point-tracker.xlsx
@@ -183,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -292,6 +292,15 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -702,7 +711,7 @@
     <row r="2">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Re-checked on 25 Sep 2026 against the code deployed to production (commit f0b36bd, 52 migrations) and against the production database. 22 completed, 9 pending. The Tracker tab carries the detail and the evidence for each row; the "After the 31 points" tab lists the work raised since this list was drawn up.</t>
+          <t>Re-checked on 25 Sep 2026 against the code deployed to production (commit f0b36bd, 52 migrations) and against the production database, then updated with Mindgate's confirmations of 25 Sep: points 1, 2, 4, 7 and 12 closed. 27 completed, 4 pending. The Tracker tab carries the detail; the "After the 31 points" tab lists the work raised since this list was drawn up.</t>
         </is>
       </c>
     </row>
@@ -713,7 +722,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C4" s="32" t="n"/>
       <c r="D4" s="32" t="n"/>
@@ -726,7 +735,7 @@
         </is>
       </c>
       <c r="B5" s="31" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C5" s="32" t="n"/>
       <c r="D5" s="32" t="n"/>
@@ -774,11 +783,11 @@
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="43" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B9" s="44" t="inlineStr">
         <is>
-          <t>Approved goals: remove the edit lock</t>
+          <t>Google Meet integration</t>
         </is>
       </c>
       <c r="C9" s="45" t="inlineStr">
@@ -788,22 +797,22 @@
       </c>
       <c r="D9" s="44" t="inlineStr">
         <is>
-          <t>Decide: should an approved growth plan be directly editable, or keep 'ask your manager to return it'? Still locked in the deployed build.</t>
+          <t>Provide Google OAuth client ID and secret for the workspace. Not configured on the box as of 25 Sep.</t>
         </is>
       </c>
       <c r="E9" s="44" t="inlineStr">
         <is>
-          <t>Mindgate — decision</t>
+          <t>Mindgate — credentials</t>
         </is>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="43" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="B10" s="44" t="inlineStr">
         <is>
-          <t>Department dropdown for KRA setup</t>
+          <t>Quarterly Connect email</t>
         </is>
       </c>
       <c r="C10" s="45" t="inlineStr">
@@ -813,22 +822,22 @@
       </c>
       <c r="D10" s="44" t="inlineStr">
         <is>
-          <t>Add a Department value to the library rows and re-publish the sheet. Checked 25 Sep: 0 of the 2,155 library rows carries a department.</t>
+          <t>Provide SMTP host, port, user and password. Still unset on production, so no mail leaves the box.</t>
         </is>
       </c>
       <c r="E10" s="44" t="inlineStr">
         <is>
-          <t>Mindgate — data</t>
+          <t>Mindgate — credentials</t>
         </is>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="43" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B11" s="44" t="inlineStr">
         <is>
-          <t>KRA unique ID</t>
+          <t>Access setup for testing</t>
         </is>
       </c>
       <c r="C11" s="45" t="inlineStr">
@@ -838,22 +847,22 @@
       </c>
       <c r="D11" s="44" t="inlineStr">
         <is>
-          <t>Answer: (a) format, e.g. SALES-SM-001; (b) unique per library row or per assigned KRA; (c) does the ID change when the KRA is edited or re-mapped; (d) what happens to the IDs already assigned. No ID field exists yet.</t>
+          <t>Mindgate is creating the employee and manager logins. Production has two logins today (hr.admin@mindgate.com, pavan.kumar@mindgate.in). Say the word if you would rather we created them.</t>
         </is>
       </c>
       <c r="E11" s="44" t="inlineStr">
         <is>
-          <t>Mindgate — decision</t>
+          <t>Mindgate — accounts</t>
         </is>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1">
       <c r="A12" s="43" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B12" s="44" t="inlineStr">
         <is>
-          <t>Google Meet integration</t>
+          <t>Quarterly connect should focus more on confirmation</t>
         </is>
       </c>
       <c r="C12" s="45" t="inlineStr">
@@ -863,147 +872,119 @@
       </c>
       <c r="D12" s="44" t="inlineStr">
         <is>
-          <t>Provide Google OAuth client ID and secret for the workspace. Not configured on the box as of 25 Sep.</t>
+          <t>Tell us what 'more confirmation' means beyond the sign-off that already exists. Adding pending sign-offs to All Approvals is small and we can do it now.</t>
         </is>
       </c>
       <c r="E12" s="44" t="inlineStr">
         <is>
-          <t>Mindgate — credentials</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="44" customHeight="1">
+          <t>Mindgate — clarify</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="43" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B13" s="44" t="inlineStr">
         <is>
-          <t>RM approval issue</t>
-        </is>
-      </c>
-      <c r="C13" s="45" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D13" s="44" t="inlineStr">
-        <is>
-          <t>Comes free with point 22. The approve path itself works and is tested; no manager with reports can sign in to exercise it.</t>
-        </is>
-      </c>
-      <c r="E13" s="44" t="inlineStr">
-        <is>
-          <t>Mindgate — accounts</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="44" customHeight="1">
+          <t>Approved goals: remove the edit lock</t>
+        </is>
+      </c>
+      <c r="C13" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D13" s="47" t="inlineStr">
+        <is>
+          <t>Closed by Mindgate 25 Sep</t>
+        </is>
+      </c>
+      <c r="E13" s="44" t="n"/>
+    </row>
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="43" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="B14" s="44" t="inlineStr">
         <is>
-          <t>KRA synchronisation</t>
-        </is>
-      </c>
-      <c r="C14" s="45" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D14" s="44" t="inlineStr">
-        <is>
-          <t>Same as point 2 — the department values on the library rows.</t>
-        </is>
-      </c>
-      <c r="E14" s="44" t="inlineStr">
-        <is>
-          <t>Mindgate — data</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="44" customHeight="1">
+          <t>Department dropdown for KRA setup</t>
+        </is>
+      </c>
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D14" s="47" t="inlineStr">
+        <is>
+          <t>Closed by Mindgate 25 Sep</t>
+        </is>
+      </c>
+      <c r="E14" s="44" t="n"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="43" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="B15" s="44" t="inlineStr">
         <is>
-          <t>Quarterly Connect email</t>
-        </is>
-      </c>
-      <c r="C15" s="45" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D15" s="44" t="inlineStr">
-        <is>
-          <t>Provide SMTP host, port, user and password. Still unset on production, so no mail leaves the box.</t>
-        </is>
-      </c>
-      <c r="E15" s="44" t="inlineStr">
-        <is>
-          <t>Mindgate — credentials</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="44" customHeight="1">
+          <t>Associate the growth path after the KRA</t>
+        </is>
+      </c>
+      <c r="C15" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D15" s="47" t="n"/>
+      <c r="E15" s="44" t="n"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
       <c r="A16" s="43" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="B16" s="44" t="inlineStr">
         <is>
-          <t>Access setup for testing</t>
-        </is>
-      </c>
-      <c r="C16" s="45" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D16" s="44" t="inlineStr">
-        <is>
-          <t>Create one manager login — somebody who actually has reports. Production has only two logins today (hr.admin@mindgate.com and pavan.kumar@mindgate.in, 0 reports). That one account unblocks point 7.</t>
-        </is>
-      </c>
-      <c r="E16" s="44" t="inlineStr">
-        <is>
-          <t>Us — needs your go-ahead</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="44" customHeight="1">
+          <t>KRA unique ID</t>
+        </is>
+      </c>
+      <c r="C16" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D16" s="47" t="inlineStr">
+        <is>
+          <t>Closed by Mindgate 25 Sep</t>
+        </is>
+      </c>
+      <c r="E16" s="44" t="n"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
       <c r="A17" s="43" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="B17" s="44" t="inlineStr">
         <is>
-          <t>Quarterly connect should focus more on confirmation</t>
-        </is>
-      </c>
-      <c r="C17" s="45" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D17" s="44" t="inlineStr">
-        <is>
-          <t>Tell us what 'more confirmation' means beyond the sign-off that already exists. Adding pending sign-offs to All Approvals is small and we can do it now.</t>
-        </is>
-      </c>
-      <c r="E17" s="44" t="inlineStr">
-        <is>
-          <t>Mindgate — clarify</t>
-        </is>
-      </c>
+          <t>KRAs always open + new-hire auto-assign</t>
+        </is>
+      </c>
+      <c r="C17" s="46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D17" s="47" t="n"/>
+      <c r="E17" s="44" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="43" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B18" s="44" t="inlineStr">
         <is>
-          <t>Associate the growth path after the KRA</t>
+          <t>RM approval issue</t>
         </is>
       </c>
       <c r="C18" s="46" t="inlineStr">
@@ -1011,24 +992,20 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D18" s="44" t="inlineStr">
-        <is>
-          <t>Tell us what 'more confirmation' means beyond sign-off. Adding pending sign-offs to All Approvals is small and we can do it now.</t>
-        </is>
-      </c>
-      <c r="E18" s="44" t="inlineStr">
-        <is>
-          <t>Mindgate — clarify</t>
-        </is>
-      </c>
+      <c r="D18" s="47" t="inlineStr">
+        <is>
+          <t>Confirmed working by Mindgate 25 Sep</t>
+        </is>
+      </c>
+      <c r="E18" s="44" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="43" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B19" s="44" t="inlineStr">
         <is>
-          <t>KRAs always open + new-hire auto-assign</t>
+          <t>ANTHROPIC_API_KEY missing in My Growth</t>
         </is>
       </c>
       <c r="C19" s="46" t="inlineStr">
@@ -1036,16 +1013,16 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D19" s="44" t="inlineStr"/>
-      <c r="E19" s="44" t="inlineStr"/>
+      <c r="D19" s="47" t="n"/>
+      <c r="E19" s="44" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="43" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B20" s="44" t="inlineStr">
         <is>
-          <t>ANTHROPIC_API_KEY missing in My Growth</t>
+          <t>KRA Library editing</t>
         </is>
       </c>
       <c r="C20" s="46" t="inlineStr">
@@ -1053,16 +1030,16 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D20" s="44" t="inlineStr"/>
-      <c r="E20" s="44" t="inlineStr"/>
+      <c r="D20" s="47" t="n"/>
+      <c r="E20" s="44" t="n"/>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="43" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B21" s="44" t="inlineStr">
         <is>
-          <t>KRA Library editing</t>
+          <t>Role / department change</t>
         </is>
       </c>
       <c r="C21" s="46" t="inlineStr">
@@ -1070,16 +1047,16 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D21" s="44" t="inlineStr"/>
-      <c r="E21" s="44" t="inlineStr"/>
+      <c r="D21" s="47" t="n"/>
+      <c r="E21" s="44" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="43" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B22" s="44" t="inlineStr">
         <is>
-          <t>Role / department change</t>
+          <t>'Select all KRAs' in My Growth</t>
         </is>
       </c>
       <c r="C22" s="46" t="inlineStr">
@@ -1087,16 +1064,16 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D22" s="44" t="inlineStr"/>
-      <c r="E22" s="44" t="inlineStr"/>
+      <c r="D22" s="47" t="n"/>
+      <c r="E22" s="44" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="43" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B23" s="44" t="inlineStr">
         <is>
-          <t>'Select all KRAs' in My Growth</t>
+          <t>KRA synchronisation</t>
         </is>
       </c>
       <c r="C23" s="46" t="inlineStr">
@@ -1104,8 +1081,12 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D23" s="44" t="inlineStr"/>
-      <c r="E23" s="44" t="inlineStr"/>
+      <c r="D23" s="47" t="inlineStr">
+        <is>
+          <t>Closed by Mindgate 25 Sep</t>
+        </is>
+      </c>
+      <c r="E23" s="44" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="43" t="n">
@@ -1121,8 +1102,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D24" s="44" t="inlineStr"/>
-      <c r="E24" s="44" t="inlineStr"/>
+      <c r="D24" s="47" t="n"/>
+      <c r="E24" s="44" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="43" t="n">
@@ -1138,8 +1119,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D25" s="44" t="inlineStr"/>
-      <c r="E25" s="44" t="inlineStr"/>
+      <c r="D25" s="47" t="n"/>
+      <c r="E25" s="44" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="43" t="n">
@@ -1155,8 +1136,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D26" s="44" t="inlineStr"/>
-      <c r="E26" s="44" t="inlineStr"/>
+      <c r="D26" s="47" t="n"/>
+      <c r="E26" s="44" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="43" t="n">
@@ -1172,8 +1153,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D27" s="44" t="inlineStr"/>
-      <c r="E27" s="44" t="inlineStr"/>
+      <c r="D27" s="47" t="n"/>
+      <c r="E27" s="44" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="43" t="n">
@@ -1189,8 +1170,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D28" s="44" t="inlineStr"/>
-      <c r="E28" s="44" t="inlineStr"/>
+      <c r="D28" s="47" t="n"/>
+      <c r="E28" s="44" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="43" t="n">
@@ -1206,8 +1187,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D29" s="44" t="inlineStr"/>
-      <c r="E29" s="44" t="inlineStr"/>
+      <c r="D29" s="47" t="n"/>
+      <c r="E29" s="44" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="43" t="n">
@@ -1223,8 +1204,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D30" s="44" t="inlineStr"/>
-      <c r="E30" s="44" t="inlineStr"/>
+      <c r="D30" s="47" t="n"/>
+      <c r="E30" s="44" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="43" t="n">
@@ -1240,8 +1221,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D31" s="44" t="inlineStr"/>
-      <c r="E31" s="44" t="inlineStr"/>
+      <c r="D31" s="47" t="n"/>
+      <c r="E31" s="44" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="43" t="n">
@@ -1257,8 +1238,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D32" s="44" t="inlineStr"/>
-      <c r="E32" s="44" t="inlineStr"/>
+      <c r="D32" s="47" t="n"/>
+      <c r="E32" s="44" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="43" t="n">
@@ -1274,8 +1255,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D33" s="44" t="inlineStr"/>
-      <c r="E33" s="44" t="inlineStr"/>
+      <c r="D33" s="47" t="n"/>
+      <c r="E33" s="44" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="43" t="n">
@@ -1291,8 +1272,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D34" s="44" t="inlineStr"/>
-      <c r="E34" s="44" t="inlineStr"/>
+      <c r="D34" s="47" t="n"/>
+      <c r="E34" s="44" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="43" t="n">
@@ -1308,8 +1289,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D35" s="44" t="inlineStr"/>
-      <c r="E35" s="44" t="inlineStr"/>
+      <c r="D35" s="47" t="n"/>
+      <c r="E35" s="44" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="43" t="n">
@@ -1325,8 +1306,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D36" s="44" t="inlineStr"/>
-      <c r="E36" s="44" t="inlineStr"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="44" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="43" t="n">
@@ -1342,8 +1323,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D37" s="44" t="inlineStr"/>
-      <c r="E37" s="44" t="inlineStr"/>
+      <c r="D37" s="47" t="n"/>
+      <c r="E37" s="44" t="n"/>
     </row>
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="43" t="n">
@@ -1359,8 +1340,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D38" s="44" t="inlineStr"/>
-      <c r="E38" s="44" t="inlineStr"/>
+      <c r="D38" s="47" t="n"/>
+      <c r="E38" s="44" t="n"/>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="43" t="n">
@@ -1376,8 +1357,8 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="D39" s="44" t="inlineStr"/>
-      <c r="E39" s="44" t="inlineStr"/>
+      <c r="D39" s="47" t="n"/>
+      <c r="E39" s="44" t="n"/>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="38" t="inlineStr">
@@ -2057,7 +2038,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Status re-checked against the code deployed to production (commit f0b36bd, 52 migrations) and against the production database, on 25 Sep 2026.</t>
+          <t>Status re-checked against the code deployed to production (commit f0b36bd, 52 migrations) and against the production database, on 25 Sep 2026. Points 1, 2, 4, 7 and 12 closed by Mindgate on 25 Sep.</t>
         </is>
       </c>
     </row>
@@ -2139,22 +2120,22 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Partly done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Phase lock IS removed: growthEditable() allows edits up to Calibration, and a RETURNED plan is editable in any phase. An APPROVED plan stays locked by design.</t>
+          <t>Closed by Mindgate 25 Sep 2026. The phase lock was already removed — growthEditable() allows edits up to Calibration and a returned plan is editable in any phase. An approved plan still has to be returned by the manager before it can be edited; Mindgate confirmed that is the wanted behaviour.</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Mindgate — decision</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Decide: should an approved growth plan be directly editable, or keep 'ask your manager to return it'?</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="H5" s="4" t="n">
@@ -2181,22 +2162,22 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Blocked on data</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Built: the KRA library is keyed on department + designation and the page has an 'All departments' filter. Live data: 0 of 2,155 library rows carry a department.</t>
+          <t>Closed by Mindgate 25 Sep 2026 — resolved through the department mapping. The KRA library is keyed on department + designation and the page filters by department. Note for the record: as of 25 Sep the 2,155 rows on production still carry no department value, so live matching falls back to designation until a sheet with departments is uploaded.</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Mindgate — data</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>Add a Department value to the library rows and re-publish the sheet.</t>
+          <t>None. Upload a library sheet carrying departments whenever you want matching to narrow by department.</t>
         </is>
       </c>
       <c r="H6" s="8" t="n">
@@ -2263,22 +2244,22 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Not built</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>No ID scheme exists. Needs four answers before any code.</t>
+          <t>Closed by Mindgate 25 Sep 2026 — the department + designation mapping identifies a KRA, so no separate unique-ID scheme is required. No ID field was built.</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Mindgate — decision</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Answer: (a) format, e.g. SALES-SM-001; (b) unique per library row or per assigned KRA; (c) does the ID change when the KRA is edited or re-mapped; (d) what happens to the 2,155 rows already loaded.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="H8" s="8" t="n">
@@ -2385,22 +2366,22 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Blocked on accounts</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>The approve path works: All Approvals currently lists sheets waiting on named managers, and the decide endpoint is covered by tests. But 0 of your 239 managers has a password, so no RM can sign in to try it.</t>
+          <t>Closed by Mindgate 25 Sep 2026 — confirmed working. All Approvals lists sheets waiting on the named manager and the decide endpoint is covered by tests; the reporting manager can approve.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Mindgate — accounts</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Comes free with point 22.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="H11" s="4" t="n"/>
@@ -2587,22 +2568,22 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Blocked on data</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Matching is department + designation first, then a company-wide fallback — never both. With 0 departments in the library it can only ever match on designation.</t>
+          <t>Closed by Mindgate 25 Sep 2026 — resolved with point 2. Matching is department + designation first, then a company-wide fallback, never both.</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Mindgate — data</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>Same as point 2.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="H16" s="8" t="n">
@@ -2989,22 +2970,22 @@
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Not built</t>
+          <t>With Mindgate</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Partly resolved. Two logins exist on production: hr.admin@mindgate.com (admin) and pavan.kumar@mindgate.in (employee role, 0 reports). There is still NO manager login with reports, so the manager approval path (point 7) cannot be exercised end to end.</t>
+          <t>Mindgate confirmed 25 Sep 2026 that the logins will be created from their side. Production has two logins today: hr.admin@mindgate.com (admin) and pavan.kumar@mindgate.in (employee role, 0 reports).</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>Us — needs your go-ahead</t>
+          <t>Mindgate — accounts</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>Create one manager login — somebody who actually has reports. That alone unblocks point 7 and lets the full submit-approve loop be demonstrated.</t>
+          <t>Create the employee and manager logins. Tell us if you would rather we created them.</t>
         </is>
       </c>
       <c r="H26" s="8" t="n">
@@ -3410,7 +3391,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Counts are formulas over the Tracker tab, so they follow it as you work. Checked against the deployed code on 24 Sep 2026.</t>
+          <t>Counts are formulas over the Tracker tab, so they follow it as you work. Checked against the deployed code on 25 Sep 2026 and updated with Mindgate's closures of the same day (points 1, 2, 4, 7 and 12).</t>
         </is>
       </c>
     </row>
@@ -3498,7 +3479,7 @@
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>Blocked on accounts</t>
+          <t>With Mindgate</t>
         </is>
       </c>
       <c r="B9" s="16">
@@ -3507,7 +3488,7 @@
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Built, cannot be tested until test logins exist.</t>
+          <t>Built; waiting on the test logins Mindgate is creating.</t>
         </is>
       </c>
     </row>
@@ -3600,7 +3581,7 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>Create one employee and one manager test login (point 22). Unblocks 7, and lets you test the approval flow end to end as the people who will use it.</t>
+          <t>Create the employee and manager test logins (point 22), so the submit-approve loop can be demonstrated end to end.</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3591,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>Decide point 1: should an approved growth plan be editable without the manager returning it?</t>
+          <t>Give us SMTP (point 17) so reminders and connect invitations actually leave the box.</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3601,7 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>Add Department values to the KRA library (points 2 and 12). Until then department matching cannot bite.</t>
+          <t>Give us the Google OAuth client ID and secret (point 5) to switch Meet links on.</t>
         </is>
       </c>
     </row>
@@ -3630,7 +3611,7 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>Fill the Career Pathing Matrix (13), and tell us what ‘more confirmation’ means for connects (31).</t>
+          <t>Tell us what ‘more confirmation’ means for quarterly connects (point 31) and we build it the same day.</t>
         </is>
       </c>
     </row>
@@ -3640,7 +3621,7 @@
       </c>
       <c r="B23" s="22" t="inlineStr">
         <is>
-          <t>Answer the four KRA unique-ID questions (4).</t>
+          <t>Confirm the new mid-year visibility (point 20) — the employee no longer sees the manager’s mid-year rating at all.</t>
         </is>
       </c>
     </row>
@@ -3650,7 +3631,7 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>Confirm the new mid-year visibility (20) — the employee no longer sees the manager’s mid-year rating at all.</t>
+          <t>Upload the suggested Career Pathing Matrix, and send prior-year ratings so Super 50 and the 9-box have history to read.</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3641,7 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>We build the last piece of 24: may a manager edit a report’s sheet during review and Save &amp; Submit?</t>
+          <t>Assign a reporting manager to the 61 employees who have none (Development 27, Application Support 22).</t>
         </is>
       </c>
     </row>
@@ -3703,14 +3684,14 @@
     <row r="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>The ten points waiting on Mindgate</t>
+          <t>The points waiting on Mindgate</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nothing on this tab can be finished by us alone.</t>
+          <t>Nothing on this tab can be finished by us alone. Points 1, 2, 4, 7 and 12 were closed by Mindgate on 25 Sep and have come off it.</t>
         </is>
       </c>
     </row>
@@ -3741,234 +3722,218 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="24" t="inlineStr">
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="48" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
-        <is>
-          <t>One employee login and one manager login on production</t>
-        </is>
-      </c>
-      <c r="C5" s="25" t="inlineStr">
-        <is>
-          <t>Only hr.admin@mindgate.com has a password; 239 managers have a role but no way in</t>
-        </is>
-      </c>
-      <c r="D5" s="24" t="inlineStr">
-        <is>
-          <t>Mindgate / us on your word</t>
-        </is>
-      </c>
-      <c r="E5" s="24" t="inlineStr"/>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="26" t="inlineStr">
-        <is>
-          <t>2, 12</t>
-        </is>
-      </c>
-      <c r="B6" s="27" t="inlineStr">
-        <is>
-          <t>A Department value on the KRA library rows</t>
-        </is>
-      </c>
-      <c r="C6" s="27" t="inlineStr">
-        <is>
-          <t>0 of 2,155 rows carry one, so matching can only use designation</t>
-        </is>
-      </c>
-      <c r="D6" s="26" t="inlineStr">
+      <c r="B5" s="48" t="inlineStr">
+        <is>
+          <t>The employee and manager logins on production</t>
+        </is>
+      </c>
+      <c r="C5" s="48" t="inlineStr">
+        <is>
+          <t>Mindgate is creating them; only hr.admin@mindgate.com and pavan.kumar@mindgate.in exist today</t>
+        </is>
+      </c>
+      <c r="D5" s="48" t="inlineStr">
+        <is>
+          <t>Mindgate — accounts</t>
+        </is>
+      </c>
+      <c r="E5" s="48" t="n"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="49" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>SMTP host, port, user, password</t>
+        </is>
+      </c>
+      <c r="C6" s="49" t="inlineStr">
+        <is>
+          <t>No mail can leave the box, so reminders and connect invitations stay in-app</t>
+        </is>
+      </c>
+      <c r="D6" s="49" t="inlineStr">
+        <is>
+          <t>Mindgate — IT</t>
+        </is>
+      </c>
+      <c r="E6" s="49" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="48" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7" s="48" t="inlineStr">
+        <is>
+          <t>Google OAuth client ID and secret</t>
+        </is>
+      </c>
+      <c r="C7" s="48" t="inlineStr">
+        <is>
+          <t>Meet cannot be connected without them</t>
+        </is>
+      </c>
+      <c r="D7" s="48" t="inlineStr">
+        <is>
+          <t>Mindgate — IT</t>
+        </is>
+      </c>
+      <c r="E7" s="48" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="49" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>What 'more confirmation' means beyond manager sign-off</t>
+        </is>
+      </c>
+      <c r="C8" s="49" t="inlineStr">
+        <is>
+          <t>Sign-off is already built</t>
+        </is>
+      </c>
+      <c r="D8" s="49" t="inlineStr">
+        <is>
+          <t>Mindgate</t>
+        </is>
+      </c>
+      <c r="E8" s="49" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="48" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="48" t="inlineStr">
+        <is>
+          <t>Rotate the Anthropic API key</t>
+        </is>
+      </c>
+      <c r="C9" s="48" t="inlineStr">
+        <is>
+          <t>Flagged repeatedly; the key is still live on the box</t>
+        </is>
+      </c>
+      <c r="D9" s="48" t="inlineStr">
+        <is>
+          <t>Mindgate — IT</t>
+        </is>
+      </c>
+      <c r="E9" s="48" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>Confirmation that the employee should never see the manager’s mid-year rating</t>
+        </is>
+      </c>
+      <c r="C10" s="49" t="inlineStr">
+        <is>
+          <t>You asked for it removed on 23 Sep; it is now hidden even after publish</t>
+        </is>
+      </c>
+      <c r="D10" s="49" t="inlineStr">
+        <is>
+          <t>Mindgate</t>
+        </is>
+      </c>
+      <c r="E10" s="49" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="48" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B11" s="48" t="inlineStr">
+        <is>
+          <t>The Career Pathing Matrix uploaded back</t>
+        </is>
+      </c>
+      <c r="C11" s="48" t="inlineStr">
+        <is>
+          <t>159 transitions are generated and downloadable; nothing has been uploaded yet</t>
+        </is>
+      </c>
+      <c r="D11" s="48" t="inlineStr">
         <is>
           <t>Mindgate — HR</t>
         </is>
       </c>
-      <c r="E6" s="26" t="inlineStr"/>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B7" s="25" t="inlineStr">
-        <is>
-          <t>Google OAuth client ID and secret</t>
-        </is>
-      </c>
-      <c r="C7" s="25" t="inlineStr">
-        <is>
-          <t>Meet cannot be connected without them</t>
-        </is>
-      </c>
-      <c r="D7" s="24" t="inlineStr">
-        <is>
-          <t>Mindgate — IT</t>
-        </is>
-      </c>
-      <c r="E7" s="24" t="inlineStr"/>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="26" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>SMTP host, port, user, password</t>
-        </is>
-      </c>
-      <c r="C8" s="27" t="inlineStr">
-        <is>
-          <t>Connect scheduling cannot send email</t>
-        </is>
-      </c>
-      <c r="D8" s="26" t="inlineStr">
-        <is>
-          <t>Mindgate — IT</t>
-        </is>
-      </c>
-      <c r="E8" s="26" t="inlineStr"/>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="inlineStr">
-        <is>
-          <t>A decision: may an approved growth plan be edited directly?</t>
-        </is>
-      </c>
-      <c r="C9" s="25" t="inlineStr">
-        <is>
-          <t>Today it must be returned by the manager first</t>
-        </is>
-      </c>
-      <c r="D9" s="24" t="inlineStr">
-        <is>
-          <t>Mindgate</t>
-        </is>
-      </c>
-      <c r="E9" s="24" t="inlineStr"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B10" s="27" t="inlineStr">
-        <is>
-          <t>Four answers on KRA unique IDs — format, scope, regeneration, back-fill</t>
-        </is>
-      </c>
-      <c r="C10" s="27" t="inlineStr">
-        <is>
-          <t>No scheme can be chosen without them</t>
-        </is>
-      </c>
-      <c r="D10" s="26" t="inlineStr">
-        <is>
-          <t>Mindgate</t>
-        </is>
-      </c>
-      <c r="E10" s="26" t="inlineStr"/>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="24" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="inlineStr">
-        <is>
-          <t>Career Pathing Matrix content</t>
-        </is>
-      </c>
-      <c r="C11" s="25" t="inlineStr">
-        <is>
-          <t>The matrix is empty, so Aspiring Career has no target roles to offer</t>
-        </is>
-      </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="E11" s="48" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>Prior-year annual ratings</t>
+        </is>
+      </c>
+      <c r="C12" s="49" t="inlineStr">
+        <is>
+          <t>Super 50 needs three years of history and the derived 9-box needs published ratings; there are none</t>
+        </is>
+      </c>
+      <c r="D12" s="49" t="inlineStr">
         <is>
           <t>Mindgate — HR</t>
         </is>
       </c>
-      <c r="E11" s="24" t="inlineStr"/>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="B12" s="27" t="inlineStr">
-        <is>
-          <t>What 'more confirmation' means beyond manager sign-off</t>
-        </is>
-      </c>
-      <c r="C12" s="27" t="inlineStr">
-        <is>
-          <t>Sign-off is already built</t>
-        </is>
-      </c>
-      <c r="D12" s="26" t="inlineStr">
-        <is>
-          <t>Mindgate</t>
-        </is>
-      </c>
-      <c r="E12" s="26" t="inlineStr"/>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="24" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="inlineStr">
-        <is>
-          <t>Rotate the Anthropic API key</t>
-        </is>
-      </c>
-      <c r="C13" s="25" t="inlineStr">
-        <is>
-          <t>Flagged repeatedly; the key is live on the box</t>
-        </is>
-      </c>
-      <c r="D13" s="24" t="inlineStr">
-        <is>
-          <t>Mindgate — IT</t>
-        </is>
-      </c>
-      <c r="E13" s="24" t="inlineStr"/>
+      <c r="E12" s="49" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B13" s="48" t="inlineStr">
+        <is>
+          <t>A reporting manager for 61 employees</t>
+        </is>
+      </c>
+      <c r="C13" s="48" t="inlineStr">
+        <is>
+          <t>Development 27, Application Support 22 — their KRAs have nobody to approve them</t>
+        </is>
+      </c>
+      <c r="D13" s="48" t="inlineStr">
+        <is>
+          <t>Mindgate — HR</t>
+        </is>
+      </c>
+      <c r="E13" s="48" t="n"/>
     </row>
     <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="B14" s="25" t="inlineStr">
-        <is>
-          <t>Confirmation that the employee should never see the manager’s mid-year rating</t>
-        </is>
-      </c>
-      <c r="C14" s="25" t="inlineStr">
-        <is>
-          <t>You asked for it removed on 23 Sep; it is now hidden even after publish, which is a change from the answer we gave you</t>
-        </is>
-      </c>
-      <c r="D14" s="24" t="inlineStr">
-        <is>
-          <t>Mindgate</t>
-        </is>
-      </c>
+      <c r="A14" s="24" t="n"/>
+      <c r="B14" s="25" t="n"/>
+      <c r="C14" s="25" t="n"/>
+      <c r="D14" s="24" t="n"/>
       <c r="E14" s="24" t="n"/>
     </row>
   </sheetData>

</xml_diff>